<commit_message>
Uppdatering av figurer och diverse text
</commit_message>
<xml_diff>
--- a/Data/arbetsloshet_kommun.xlsx
+++ b/Data/arbetsloshet_kommun.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">region_kod</t>
   </si>
@@ -56,7 +56,7 @@
     <t xml:space="preserve">arbetslöshet</t>
   </si>
   <si>
-    <t xml:space="preserve">2026M04</t>
+    <t xml:space="preserve">2026M05</t>
   </si>
   <si>
     <t xml:space="preserve">2-4</t>
@@ -141,9 +141,6 @@
   </si>
   <si>
     <t xml:space="preserve">Avesta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6+</t>
   </si>
   <si>
     <t xml:space="preserve">2085</t>
@@ -530,7 +527,7 @@
         <v>14</v>
       </c>
       <c r="H2" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
@@ -559,7 +556,7 @@
         <v>14</v>
       </c>
       <c r="H3" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="I3" t="s">
         <v>15</v>
@@ -588,7 +585,7 @@
         <v>14</v>
       </c>
       <c r="H4" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="I4" t="s">
         <v>15</v>
@@ -646,7 +643,7 @@
         <v>14</v>
       </c>
       <c r="H6" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I6" t="s">
         <v>15</v>
@@ -675,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="H7" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="I7" t="s">
         <v>15</v>
@@ -733,7 +730,7 @@
         <v>14</v>
       </c>
       <c r="H9" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="I9" t="s">
         <v>15</v>
@@ -762,7 +759,7 @@
         <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="I10" t="s">
         <v>15</v>
@@ -791,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="H11" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="I11" t="s">
         <v>15</v>
@@ -820,7 +817,7 @@
         <v>14</v>
       </c>
       <c r="H12" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="I12" t="s">
         <v>36</v>
@@ -849,7 +846,7 @@
         <v>14</v>
       </c>
       <c r="H13" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -878,7 +875,7 @@
         <v>14</v>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="I14" t="s">
         <v>36</v>
@@ -907,19 +904,19 @@
         <v>14</v>
       </c>
       <c r="H15" t="n">
-        <v>6</v>
+        <v>5.7</v>
       </c>
       <c r="I15" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
         <v>44</v>
       </c>
-      <c r="B16" t="s">
-        <v>45</v>
-      </c>
       <c r="C16" t="s">
         <v>11</v>
       </c>
@@ -936,7 +933,7 @@
         <v>14</v>
       </c>
       <c r="H16" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="I16" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Diverse uppdateringar och ny version publicerad
</commit_message>
<xml_diff>
--- a/Data/arbetsloshet_kommun.xlsx
+++ b/Data/arbetsloshet_kommun.xlsx
@@ -56,7 +56,7 @@
     <t xml:space="preserve">arbetslöshet</t>
   </si>
   <si>
-    <t xml:space="preserve">2026M05</t>
+    <t xml:space="preserve">2026M06</t>
   </si>
   <si>
     <t xml:space="preserve">2-4</t>
@@ -527,7 +527,7 @@
         <v>14</v>
       </c>
       <c r="H2" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
@@ -556,7 +556,7 @@
         <v>14</v>
       </c>
       <c r="H3" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="I3" t="s">
         <v>15</v>
@@ -585,7 +585,7 @@
         <v>14</v>
       </c>
       <c r="H4" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="I4" t="s">
         <v>15</v>
@@ -614,7 +614,7 @@
         <v>14</v>
       </c>
       <c r="H5" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="I5" t="s">
         <v>15</v>
@@ -643,7 +643,7 @@
         <v>14</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="I6" t="s">
         <v>15</v>
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="H7" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="I7" t="s">
         <v>15</v>
@@ -701,7 +701,7 @@
         <v>14</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I8" t="s">
         <v>15</v>
@@ -730,7 +730,7 @@
         <v>14</v>
       </c>
       <c r="H9" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="I9" t="s">
         <v>15</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="I11" t="s">
         <v>15</v>
@@ -817,7 +817,7 @@
         <v>14</v>
       </c>
       <c r="H12" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="I12" t="s">
         <v>36</v>
@@ -846,7 +846,7 @@
         <v>14</v>
       </c>
       <c r="H13" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -875,7 +875,7 @@
         <v>14</v>
       </c>
       <c r="H14" t="n">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="I14" t="s">
         <v>36</v>
@@ -904,7 +904,7 @@
         <v>14</v>
       </c>
       <c r="H15" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="I15" t="s">
         <v>36</v>

</xml_diff>